<commit_message>
proposal: restructured v2 proposal, updated seminar deck, failing-query deep dive
- research_proposal_v2.tex/.pdf: plain-language restructure per advisor outline
  (glossary, three goals, RQ1-3, phases 1-4 with problem/approach/evaluation,
  Algorithm 1, three-semester Gantt); 13 follow-up comments applied
- research_proposal.tex/.pdf: 25-page expanded version kept as is
- verified bibliographies (references, refs_rag, refs_geometry, refs_new) and
  plainnat-hyphen.bst (plain hyphens in page ranges)
- figures/ and proposal_figures.py: trilateration, triangle, gradient, sweeps
- deep_dive_failing_queries.py -> H2_failing_deep_dive.xlsx (58 failing queries)
- seminar_presentation.pptx rebuilt to match v2 (15 slides)
- remove outdated meeting_prep PDFs

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proposal/H2_results.xlsx
+++ b/proposal/H2_results.xlsx
@@ -1296,7 +1296,7 @@
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>d(Q,GT) ≈ 0.22 avg  vs  d(C,GT) ≈ 0.10  and  d(Q,C) ≈ 0.18. Queries sit noticeably further from their relevant documents.</t>
+          <t>d(Q,GT) ≈ 0.17 avg  vs  d(C,GT) ≈ 0.10  and  d(Q,C) ≈ 0.17. Queries sit noticeably further from their relevant documents.</t>
         </is>
       </c>
     </row>
@@ -11968,7 +11968,7 @@
       </c>
       <c r="E6" s="83" t="inlineStr">
         <is>
-          <t>Top-1 = 17.9%   Avg. GT Rank = 17.6
+          <t>Top-1 = 14.8%   Avg. GT Rank = 9.87
 Worst overall. Centroid is not a reliable proxy for the query.</t>
         </is>
       </c>

</xml_diff>